<commit_message>
quick save before some changes
</commit_message>
<xml_diff>
--- a/PV_ICE/baselines/SupportingMaterial/Manual Files/Inverter_Gallium_Calcs.xlsx
+++ b/PV_ICE/baselines/SupportingMaterial/Manual Files/Inverter_Gallium_Calcs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hmirletz\Documents\GitHub\PV_ICE\PV_ICE\baselines\SupportingMaterial\Manual Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10AD4139-A07E-493C-B61C-73C7F0854806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{898D25E6-5F9D-4382-A9CF-FCE690525C40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28575" yWindow="1095" windowWidth="26715" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28590" yWindow="4395" windowWidth="24915" windowHeight="10680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="97">
   <si>
     <t>year</t>
   </si>
@@ -55,16 +55,10 @@
     <t>Chips per inverter [#/inverter type]</t>
   </si>
   <si>
-    <t>Inverter Type</t>
-  </si>
-  <si>
     <t>Source2</t>
   </si>
   <si>
     <t>Notes2</t>
-  </si>
-  <si>
-    <t>GaN FET/ 10 kW single phase</t>
   </si>
   <si>
     <t>GaN FET/ 1.6kW microinverter</t>
@@ -415,26 +409,82 @@
     <t>see google sheet for avg calc</t>
   </si>
   <si>
-    <t>Micro</t>
-  </si>
-  <si>
-    <t>String</t>
-  </si>
-  <si>
-    <t>Utility</t>
-  </si>
-  <si>
     <t>[g/FET]</t>
   </si>
   <si>
     <t>% GaN HEMT in PV application market</t>
+  </si>
+  <si>
+    <t>Silvana counted 6 in the circuit diagram</t>
+  </si>
+  <si>
+    <t>GaN FET/ 10 kW single phase with Battery</t>
+  </si>
+  <si>
+    <t>*Heather will go back and inventory all the GaN TI ref designs adding # of phases and Voltage</t>
+  </si>
+  <si>
+    <t>SELECTED AS REPRESENTATIVE DESIGN</t>
+  </si>
+  <si>
+    <t>MICRO</t>
+  </si>
+  <si>
+    <t>UTILITY</t>
+  </si>
+  <si>
+    <t>STRING</t>
+  </si>
+  <si>
+    <t># of Phases</t>
+  </si>
+  <si>
+    <t>500 V</t>
+  </si>
+  <si>
+    <t>600, 800, 1000 V</t>
+  </si>
+  <si>
+    <t>Voltages [V]</t>
+  </si>
+  <si>
+    <t>Inverter Description</t>
+  </si>
+  <si>
+    <t>60 Vdc, 240 Vac</t>
+  </si>
+  <si>
+    <t>*check for a material value</t>
+  </si>
+  <si>
+    <t>Micro [g/inverter]</t>
+  </si>
+  <si>
+    <t>String [g/inverter]</t>
+  </si>
+  <si>
+    <t>Utility [g/inverter]</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/tool/TIDA-010949</t>
+  </si>
+  <si>
+    <t>80 V</t>
+  </si>
+  <si>
+    <t>600W solar power optimizer reference design based on GaN with wired and wireless communication</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <numFmts count="3">
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="0.000%"/>
+    <numFmt numFmtId="171" formatCode="0.000000000E+00"/>
+  </numFmts>
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -509,13 +559,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="9">
@@ -613,7 +677,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -625,15 +689,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -643,6 +703,28 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -967,7 +1049,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V112"/>
+  <dimension ref="A1:Y112"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.81640625" bestFit="1" customWidth="1"/>
@@ -975,17 +1057,20 @@
     <col min="3" max="3" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="1.453125" customWidth="1"/>
     <col min="7" max="7" width="15.81640625" customWidth="1"/>
-    <col min="8" max="8" width="36" customWidth="1"/>
-    <col min="11" max="11" width="1.08984375" customWidth="1"/>
-    <col min="12" max="12" width="12.08984375" customWidth="1"/>
-    <col min="13" max="13" width="4.36328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.08984375" customWidth="1"/>
-    <col min="15" max="15" width="16.90625" customWidth="1"/>
-    <col min="16" max="16" width="1.1796875" customWidth="1"/>
-    <col min="17" max="19" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="8.90625" customWidth="1"/>
-    <col min="21" max="22" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="36" customWidth="1"/>
+    <col min="11" max="11" width="17" style="4" customWidth="1"/>
+    <col min="14" max="14" width="1.08984375" customWidth="1"/>
+    <col min="15" max="15" width="12.08984375" customWidth="1"/>
+    <col min="16" max="16" width="4.36328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.08984375" customWidth="1"/>
+    <col min="18" max="18" width="16.90625" customWidth="1"/>
+    <col min="19" max="19" width="1.1796875" customWidth="1"/>
+    <col min="20" max="22" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="8.90625" customWidth="1"/>
+    <col min="24" max="25" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="18.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -993,10 +1078,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>2</v>
@@ -1008,43 +1093,43 @@
         <v>4</v>
       </c>
       <c r="H1" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="K1" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="R1" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="O1" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>79</v>
-      </c>
       <c r="T1" s="3" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.35">
@@ -1122,57 +1207,62 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>2005</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>2006</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>2007</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>2008</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>2009</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>2010</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>2011</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>2012</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>2013</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>2014</v>
       </c>
-    </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="G26" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="H26" s="19"/>
+      <c r="I26" s="19"/>
+    </row>
+    <row r="27" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>2015</v>
       </c>
@@ -1180,16 +1270,16 @@
         <v>5.12</v>
       </c>
       <c r="C27" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>2016</v>
       </c>
@@ -1198,297 +1288,261 @@
         <v>1E-4</v>
       </c>
       <c r="C28" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E28" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>2017</v>
       </c>
-      <c r="L29" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="O29" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="30" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>2018</v>
       </c>
-      <c r="L30" s="18">
-        <v>2.3529411764705885E-3</v>
-      </c>
-      <c r="M30" t="s">
+      <c r="O30" s="14">
+        <v>3.1809145129224651E-5</v>
+      </c>
+      <c r="P30" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>72</v>
+      </c>
+      <c r="R30" t="s">
         <v>73</v>
       </c>
-      <c r="N30" t="s">
-        <v>74</v>
-      </c>
-      <c r="O30" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q30">
-        <f>$B$37*$G$35*L30</f>
-        <v>7.9529411764705882E-7</v>
-      </c>
-      <c r="R30">
-        <f>$B$37*$G$34*L30</f>
-        <v>4.7717647058823531E-7</v>
-      </c>
-      <c r="S30">
-        <f>$B$37*$G$36*L30</f>
-        <v>1.5905882352941175E-7</v>
-      </c>
       <c r="T30">
-        <f>ROUND(Q30,6)</f>
-        <v>9.9999999999999995E-7</v>
+        <f>$B$37*$G$35*O30</f>
+        <v>1.0751491053677931E-8</v>
       </c>
       <c r="U30">
-        <f>ROUND(R30,7)</f>
-        <v>4.9999999999999998E-7</v>
+        <f>$B$37*$G$34*O30</f>
+        <v>6.4508946322067582E-9</v>
       </c>
       <c r="V30">
-        <f>ROUND(S30,7)</f>
-        <v>1.9999999999999999E-7</v>
-      </c>
-    </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
+        <f>$B$37*$G$36*O30</f>
+        <v>6.4508946322067582E-9</v>
+      </c>
+      <c r="W30" s="29"/>
+      <c r="X30" s="29"/>
+      <c r="Y30" s="29"/>
+    </row>
+    <row r="31" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>2019</v>
       </c>
-      <c r="L31" s="18">
-        <v>1.9138755980861245E-3</v>
-      </c>
-      <c r="M31" t="s">
+      <c r="O31" s="14">
+        <v>3.0434451799436964E-5</v>
+      </c>
+      <c r="P31" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>72</v>
+      </c>
+      <c r="R31" t="s">
         <v>73</v>
       </c>
-      <c r="N31" t="s">
-        <v>74</v>
-      </c>
-      <c r="O31" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q31">
-        <f t="shared" ref="Q31:Q40" si="0">$B$37*$G$35*L31</f>
-        <v>6.4688995215310997E-7</v>
-      </c>
-      <c r="R31">
-        <f t="shared" ref="R31:R40" si="1">$B$37*$G$34*L31</f>
-        <v>3.8813397129186598E-7</v>
-      </c>
-      <c r="S31">
-        <f t="shared" ref="S31:S40" si="2">$B$37*$G$36*L31</f>
-        <v>1.2937799043062199E-7</v>
-      </c>
       <c r="T31">
-        <f t="shared" ref="T31:T40" si="3">ROUND(Q31,6)</f>
-        <v>9.9999999999999995E-7</v>
+        <f t="shared" ref="T31:T40" si="0">$B$37*$G$35*O31</f>
+        <v>1.0286844708209693E-8</v>
       </c>
       <c r="U31">
-        <f>ROUND(R31,7)</f>
-        <v>3.9999999999999998E-7</v>
+        <f t="shared" ref="U31:U40" si="1">$B$37*$G$34*O31</f>
+        <v>6.1721068249258155E-9</v>
       </c>
       <c r="V31">
-        <f t="shared" ref="V31:V34" si="4">ROUND(S31,7)</f>
-        <v>9.9999999999999995E-8</v>
-      </c>
-    </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
+        <f t="shared" ref="V31:V40" si="2">$B$37*$G$36*O31</f>
+        <v>6.1721068249258155E-9</v>
+      </c>
+      <c r="W31" s="29"/>
+      <c r="X31" s="29"/>
+      <c r="Y31" s="29"/>
+    </row>
+    <row r="32" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>2020</v>
       </c>
-      <c r="L32" s="18">
-        <v>3.3018867924528299E-3</v>
-      </c>
-      <c r="M32" t="s">
+      <c r="O32" s="14">
+        <v>5.4192149880003095E-5</v>
+      </c>
+      <c r="P32" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>72</v>
+      </c>
+      <c r="R32" t="s">
         <v>73</v>
       </c>
-      <c r="N32" t="s">
-        <v>74</v>
-      </c>
-      <c r="O32" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q32">
+      <c r="T32">
         <f t="shared" si="0"/>
-        <v>1.1160377358490565E-6</v>
-      </c>
-      <c r="R32">
+        <v>1.8316946659441044E-8</v>
+      </c>
+      <c r="U32">
         <f t="shared" si="1"/>
-        <v>6.6962264150943376E-7</v>
-      </c>
-      <c r="S32">
+        <v>1.0990167995664626E-8</v>
+      </c>
+      <c r="V32">
         <f t="shared" si="2"/>
-        <v>2.2320754716981128E-7</v>
-      </c>
-      <c r="T32">
-        <f t="shared" si="3"/>
-        <v>9.9999999999999995E-7</v>
-      </c>
-      <c r="U32">
-        <f t="shared" ref="U31:U40" si="5">ROUND(R32,6)</f>
-        <v>9.9999999999999995E-7</v>
-      </c>
-      <c r="V32">
-        <f t="shared" si="4"/>
-        <v>1.9999999999999999E-7</v>
-      </c>
-    </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
+        <v>1.0990167995664626E-8</v>
+      </c>
+      <c r="W32" s="29"/>
+      <c r="X32" s="29"/>
+      <c r="Y32" s="29"/>
+    </row>
+    <row r="33" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>2021</v>
       </c>
-      <c r="G33" s="16">
+      <c r="G33" s="12">
         <v>0</v>
       </c>
-      <c r="H33" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="I33" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="L33" s="18">
-        <v>3.8194444444444448E-3</v>
-      </c>
-      <c r="M33" t="s">
+      <c r="H33" s="12"/>
+      <c r="I33" s="12"/>
+      <c r="J33" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="K33" s="21"/>
+      <c r="L33" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="O33" s="14">
+        <v>8.058017727639001E-5</v>
+      </c>
+      <c r="P33" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>72</v>
+      </c>
+      <c r="R33" t="s">
         <v>73</v>
       </c>
-      <c r="N33" t="s">
-        <v>74</v>
-      </c>
-      <c r="O33" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q33">
+      <c r="T33">
         <f t="shared" si="0"/>
-        <v>1.2909722222222223E-6</v>
-      </c>
-      <c r="R33">
+        <v>2.7236099919419822E-8</v>
+      </c>
+      <c r="U33">
         <f t="shared" si="1"/>
-        <v>7.7458333333333326E-7</v>
-      </c>
-      <c r="S33">
+        <v>1.6341659951651891E-8</v>
+      </c>
+      <c r="V33">
         <f t="shared" si="2"/>
-        <v>2.5819444444444442E-7</v>
-      </c>
-      <c r="T33">
-        <f t="shared" si="3"/>
-        <v>9.9999999999999995E-7</v>
-      </c>
-      <c r="U33">
-        <f t="shared" si="5"/>
-        <v>9.9999999999999995E-7</v>
-      </c>
-      <c r="V33">
-        <f t="shared" si="4"/>
-        <v>2.9999999999999999E-7</v>
-      </c>
-    </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
+        <v>1.6341659951651891E-8</v>
+      </c>
+      <c r="W33" s="29"/>
+      <c r="X33" s="29"/>
+      <c r="Y33" s="29"/>
+    </row>
+    <row r="34" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>2022</v>
       </c>
       <c r="G34">
         <v>6</v>
       </c>
-      <c r="H34" t="s">
-        <v>8</v>
+      <c r="H34">
+        <v>1</v>
       </c>
       <c r="I34" t="s">
-        <v>11</v>
-      </c>
-      <c r="L34" s="18">
-        <v>6.8459657701711489E-3</v>
-      </c>
-      <c r="M34" t="s">
+        <v>85</v>
+      </c>
+      <c r="J34" t="s">
+        <v>78</v>
+      </c>
+      <c r="K34" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="L34" t="s">
+        <v>9</v>
+      </c>
+      <c r="O34" s="14">
+        <v>1.9553072625698323E-4</v>
+      </c>
+      <c r="P34" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>72</v>
+      </c>
+      <c r="R34" t="s">
         <v>73</v>
       </c>
-      <c r="N34" t="s">
-        <v>74</v>
-      </c>
-      <c r="O34" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q34">
+      <c r="T34">
         <f t="shared" si="0"/>
-        <v>2.3139364303178481E-6</v>
-      </c>
-      <c r="R34">
+        <v>6.6089385474860326E-8</v>
+      </c>
+      <c r="U34">
         <f t="shared" si="1"/>
-        <v>1.3883618581907089E-6</v>
-      </c>
-      <c r="S34">
+        <v>3.9653631284916192E-8</v>
+      </c>
+      <c r="V34">
         <f t="shared" si="2"/>
-        <v>4.6278728606356959E-7</v>
-      </c>
-      <c r="T34">
-        <f t="shared" si="3"/>
-        <v>1.9999999999999999E-6</v>
-      </c>
-      <c r="U34">
-        <f t="shared" si="5"/>
-        <v>9.9999999999999995E-7</v>
-      </c>
-      <c r="V34">
-        <f t="shared" si="4"/>
-        <v>4.9999999999999998E-7</v>
-      </c>
-    </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
+        <v>3.9653631284916192E-8</v>
+      </c>
+      <c r="W34" s="29"/>
+      <c r="X34" s="29"/>
+      <c r="Y34" s="29"/>
+    </row>
+    <row r="35" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>2023</v>
       </c>
       <c r="G35">
         <v>10</v>
       </c>
-      <c r="H35" t="s">
+      <c r="I35" t="s">
+        <v>89</v>
+      </c>
+      <c r="J35" t="s">
+        <v>7</v>
+      </c>
+      <c r="K35" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="L35" t="s">
         <v>9</v>
       </c>
-      <c r="I35" t="s">
-        <v>11</v>
-      </c>
-      <c r="L35" s="18">
-        <v>9.6078431372549032E-3</v>
-      </c>
-      <c r="M35" t="s">
+      <c r="O35" s="14">
+        <v>3.3690869086908695E-4</v>
+      </c>
+      <c r="P35" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>72</v>
+      </c>
+      <c r="R35" t="s">
         <v>73</v>
       </c>
-      <c r="N35" t="s">
-        <v>74</v>
-      </c>
-      <c r="O35" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q35">
+      <c r="T35">
         <f t="shared" si="0"/>
-        <v>3.2474509803921571E-6</v>
-      </c>
-      <c r="R35">
+        <v>1.1387513751375138E-7</v>
+      </c>
+      <c r="U35">
         <f t="shared" si="1"/>
-        <v>1.948470588235294E-6</v>
-      </c>
-      <c r="S35">
+        <v>6.8325082508250822E-8</v>
+      </c>
+      <c r="V35">
         <f t="shared" si="2"/>
-        <v>6.4949019607843133E-7</v>
-      </c>
-      <c r="T35">
-        <f t="shared" si="3"/>
-        <v>3.0000000000000001E-6</v>
-      </c>
-      <c r="U35">
-        <f t="shared" si="5"/>
-        <v>1.9999999999999999E-6</v>
-      </c>
-      <c r="V35">
-        <f t="shared" ref="V31:V40" si="6">ROUND(S35,6)</f>
-        <v>9.9999999999999995E-7</v>
-      </c>
-    </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
+        <v>6.8325082508250822E-8</v>
+      </c>
+      <c r="W35" s="29"/>
+      <c r="X35" s="29"/>
+      <c r="Y35" s="29"/>
+    </row>
+    <row r="36" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>2024</v>
       </c>
@@ -1496,61 +1550,64 @@
         <v>3.3799999999999997E-2</v>
       </c>
       <c r="C36" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D36" t="s">
         <v>3</v>
       </c>
       <c r="E36" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G36">
-        <v>2</v>
-      </c>
-      <c r="H36" t="s">
-        <v>10</v>
-      </c>
-      <c r="I36" t="s">
-        <v>11</v>
-      </c>
-      <c r="L36" s="18">
-        <v>1.2673611111111111E-2</v>
+        <v>6</v>
+      </c>
+      <c r="H36">
+        <v>3</v>
+      </c>
+      <c r="I36" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="J36" t="s">
+        <v>8</v>
+      </c>
+      <c r="K36" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="L36" t="s">
+        <v>9</v>
       </c>
       <c r="M36" t="s">
+        <v>77</v>
+      </c>
+      <c r="O36" s="14">
+        <v>4.8114948589506984E-4</v>
+      </c>
+      <c r="P36" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>72</v>
+      </c>
+      <c r="R36" t="s">
         <v>73</v>
       </c>
-      <c r="N36" t="s">
-        <v>74</v>
-      </c>
-      <c r="O36" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q36">
+      <c r="T36">
         <f t="shared" si="0"/>
-        <v>4.2836805555555554E-6</v>
-      </c>
-      <c r="R36">
+        <v>1.6262852623253359E-7</v>
+      </c>
+      <c r="U36">
         <f t="shared" si="1"/>
-        <v>2.5702083333333329E-6</v>
-      </c>
-      <c r="S36">
+        <v>9.7577115739520148E-8</v>
+      </c>
+      <c r="V36">
         <f t="shared" si="2"/>
-        <v>8.5673611111111104E-7</v>
-      </c>
-      <c r="T36">
-        <f t="shared" si="3"/>
-        <v>3.9999999999999998E-6</v>
-      </c>
-      <c r="U36">
-        <f t="shared" si="5"/>
-        <v>3.0000000000000001E-6</v>
-      </c>
-      <c r="V36">
-        <f t="shared" si="6"/>
-        <v>9.9999999999999995E-7</v>
-      </c>
-    </row>
-    <row r="37" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.35">
+        <v>9.7577115739520148E-8</v>
+      </c>
+      <c r="W36" s="29"/>
+      <c r="X36" s="29"/>
+      <c r="Y36" s="29"/>
+    </row>
+    <row r="37" spans="1:25" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>2025</v>
       </c>
@@ -1559,204 +1616,181 @@
         <v>3.3799999999999995E-5</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="L37" s="19">
-        <v>1.6773162939297124E-2</v>
-      </c>
-      <c r="M37" t="s">
+        <v>75</v>
+      </c>
+      <c r="H37" s="1">
+        <v>1</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="K37" s="22"/>
+      <c r="M37" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="O37" s="15">
+        <v>6.5715358618099887E-4</v>
+      </c>
+      <c r="P37" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>72</v>
+      </c>
+      <c r="R37" t="s">
         <v>73</v>
       </c>
-      <c r="N37" t="s">
-        <v>74</v>
-      </c>
-      <c r="O37" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q37">
+      <c r="T37">
         <f t="shared" si="0"/>
-        <v>5.6693290734824276E-6</v>
-      </c>
-      <c r="R37">
+        <v>2.2211791212917761E-7</v>
+      </c>
+      <c r="U37">
         <f t="shared" si="1"/>
-        <v>3.4015974440894562E-6</v>
-      </c>
-      <c r="S37">
+        <v>1.3327074727750656E-7</v>
+      </c>
+      <c r="V37">
         <f t="shared" si="2"/>
-        <v>1.1338658146964855E-6</v>
-      </c>
-      <c r="T37">
-        <f t="shared" si="3"/>
-        <v>6.0000000000000002E-6</v>
-      </c>
-      <c r="U37">
-        <f t="shared" si="5"/>
-        <v>3.0000000000000001E-6</v>
-      </c>
-      <c r="V37">
-        <f t="shared" si="6"/>
-        <v>9.9999999999999995E-7</v>
-      </c>
-    </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
+        <v>1.3327074727750656E-7</v>
+      </c>
+      <c r="W37" s="29"/>
+      <c r="X37" s="29"/>
+      <c r="Y37" s="29"/>
+    </row>
+    <row r="38" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>2026</v>
       </c>
-      <c r="L38" s="18">
-        <v>2.2962962962962963E-2</v>
-      </c>
-      <c r="M38" t="s">
+      <c r="O38" s="14">
+        <v>9.1846409101682864E-4</v>
+      </c>
+      <c r="P38" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>72</v>
+      </c>
+      <c r="R38" t="s">
         <v>73</v>
       </c>
-      <c r="N38" t="s">
-        <v>74</v>
-      </c>
-      <c r="O38" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q38">
+      <c r="T38">
         <f t="shared" si="0"/>
-        <v>7.7614814814814808E-6</v>
-      </c>
-      <c r="R38">
+        <v>3.1044086276368805E-7</v>
+      </c>
+      <c r="U38">
         <f t="shared" si="1"/>
-        <v>4.656888888888888E-6</v>
-      </c>
-      <c r="S38">
+        <v>1.8626451765821281E-7</v>
+      </c>
+      <c r="V38">
         <f t="shared" si="2"/>
-        <v>1.552296296296296E-6</v>
-      </c>
-      <c r="T38">
-        <f t="shared" si="3"/>
-        <v>7.9999999999999996E-6</v>
-      </c>
-      <c r="U38">
-        <f t="shared" si="5"/>
-        <v>5.0000000000000004E-6</v>
-      </c>
-      <c r="V38">
-        <f t="shared" si="6"/>
-        <v>1.9999999999999999E-6</v>
-      </c>
-    </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
+        <v>1.8626451765821281E-7</v>
+      </c>
+      <c r="W38" s="29"/>
+      <c r="X38" s="29"/>
+      <c r="Y38" s="29"/>
+    </row>
+    <row r="39" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>2027</v>
       </c>
-      <c r="L39" s="18">
-        <v>2.524271844660194E-2</v>
-      </c>
-      <c r="M39" t="s">
+      <c r="O39" s="14">
+        <v>1.028306683993446E-3</v>
+      </c>
+      <c r="P39" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>72</v>
+      </c>
+      <c r="R39" t="s">
         <v>73</v>
       </c>
-      <c r="N39" t="s">
-        <v>74</v>
-      </c>
-      <c r="O39" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q39">
+      <c r="T39">
         <f t="shared" si="0"/>
-        <v>8.532038834951455E-6</v>
-      </c>
-      <c r="R39">
+        <v>3.4756765918978473E-7</v>
+      </c>
+      <c r="U39">
         <f t="shared" si="1"/>
-        <v>5.1192233009708728E-6</v>
-      </c>
-      <c r="S39">
+        <v>2.085405955138708E-7</v>
+      </c>
+      <c r="V39">
         <f t="shared" si="2"/>
-        <v>1.7064077669902909E-6</v>
-      </c>
-      <c r="T39">
-        <f t="shared" si="3"/>
-        <v>9.0000000000000002E-6</v>
-      </c>
-      <c r="U39">
-        <f t="shared" si="5"/>
-        <v>5.0000000000000004E-6</v>
-      </c>
-      <c r="V39">
-        <f t="shared" si="6"/>
-        <v>1.9999999999999999E-6</v>
-      </c>
-    </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
+        <v>2.085405955138708E-7</v>
+      </c>
+      <c r="W39" s="29"/>
+      <c r="X39" s="29"/>
+      <c r="Y39" s="29"/>
+    </row>
+    <row r="40" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>2028</v>
       </c>
-      <c r="L40" s="20">
-        <v>2.8853754940711459E-2</v>
-      </c>
-      <c r="M40" t="s">
+      <c r="O40" s="16">
+        <v>1.1831442463533224E-3</v>
+      </c>
+      <c r="P40" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>72</v>
+      </c>
+      <c r="R40" t="s">
         <v>73</v>
       </c>
-      <c r="N40" t="s">
-        <v>74</v>
-      </c>
-      <c r="O40" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q40">
+      <c r="T40">
         <f t="shared" si="0"/>
-        <v>9.7525691699604717E-6</v>
-      </c>
-      <c r="R40">
+        <v>3.9990275526742293E-7</v>
+      </c>
+      <c r="U40">
         <f t="shared" si="1"/>
-        <v>5.8515415019762829E-6</v>
-      </c>
-      <c r="S40">
+        <v>2.3994165316045375E-7</v>
+      </c>
+      <c r="V40">
         <f t="shared" si="2"/>
-        <v>1.9505138339920944E-6</v>
-      </c>
-      <c r="T40">
-        <f t="shared" si="3"/>
-        <v>1.0000000000000001E-5</v>
-      </c>
-      <c r="U40">
-        <f t="shared" si="5"/>
-        <v>6.0000000000000002E-6</v>
-      </c>
-      <c r="V40">
-        <f t="shared" si="6"/>
-        <v>1.9999999999999999E-6</v>
-      </c>
-    </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
+        <v>2.3994165316045375E-7</v>
+      </c>
+      <c r="W40" s="29"/>
+      <c r="X40" s="29"/>
+      <c r="Y40" s="29"/>
+    </row>
+    <row r="41" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>2029</v>
       </c>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>2030</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>2031</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>2032</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>2033</v>
       </c>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>2034</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>2035</v>
       </c>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>2036</v>
       </c>
@@ -2084,9 +2118,10 @@
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="I33" r:id="rId1" display="https://doi.org/10.1016/j.resconrec.2023.107391" xr:uid="{C91B04C4-6F06-46FC-95C3-9BE3E8D63B79}"/>
+    <hyperlink ref="L33" r:id="rId1" display="https://doi.org/10.1016/j.resconrec.2023.107391" xr:uid="{C91B04C4-6F06-46FC-95C3-9BE3E8D63B79}"/>
     <hyperlink ref="D27" r:id="rId2" display="https://doi.org/10.1016/j.resconrec.2023.107391" xr:uid="{46E41433-83E9-41D0-81BF-194345B4E180}"/>
     <hyperlink ref="D28" r:id="rId3" display="https://doi.org/10.1016/j.resconrec.2023.107391" xr:uid="{834D0FB7-3EFD-43D3-9B68-EB35F321DE1A}"/>
+    <hyperlink ref="M37" r:id="rId4" xr:uid="{7B120840-CD9C-400D-9838-2232DE726815}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2094,58 +2129,61 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B730B5FD-02A7-4220-AE14-32AAECAEAC50}">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="5.81640625" customWidth="1"/>
+    <col min="2" max="2" width="10.81640625" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="9.36328125" customWidth="1"/>
     <col min="5" max="5" width="14.7265625" customWidth="1"/>
     <col min="6" max="6" width="11.26953125" customWidth="1"/>
-    <col min="7" max="7" width="4.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.08984375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="6.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B2" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B2" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" t="s">
         <v>56</v>
       </c>
-      <c r="C3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>58</v>
       </c>
-      <c r="E3" t="s">
-        <v>60</v>
-      </c>
       <c r="F3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G3" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="H3" t="s">
         <v>56</v>
       </c>
-      <c r="G3" t="s">
-        <v>57</v>
-      </c>
-      <c r="H3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2018</v>
       </c>
@@ -2162,20 +2200,20 @@
         <f>SUM(B4:D4)</f>
         <v>16.099999999999998</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <f>B4/$E4</f>
         <v>2.4844720496894415E-2</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="25">
         <f t="shared" ref="G4:H4" si="0">C4/$E4</f>
         <v>0</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="6">
         <f t="shared" si="0"/>
         <v>0.97515527950310565</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2019</v>
       </c>
@@ -2189,23 +2227,23 @@
         <v>16.5</v>
       </c>
       <c r="E5">
-        <f t="shared" ref="E5:E15" si="1">SUM(B5:D5)</f>
+        <f t="shared" ref="E5:E14" si="1">SUM(B5:D5)</f>
         <v>17.11</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="7">
         <f t="shared" ref="F5:F14" si="2">B5/$E5</f>
         <v>3.5067212156633547E-2</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="26">
         <f t="shared" ref="G5:G14" si="3">C5/$E5</f>
         <v>5.8445353594389253E-4</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="8">
         <f t="shared" ref="H5:H14" si="4">D5/$E5</f>
         <v>0.96434833430742262</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2020</v>
       </c>
@@ -2222,20 +2260,20 @@
         <f t="shared" si="1"/>
         <v>17.22</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="7">
         <f t="shared" si="2"/>
         <v>4.065040650406504E-2</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="26">
         <f t="shared" si="3"/>
         <v>1.1614401858304297E-3</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="8">
         <f t="shared" si="4"/>
         <v>0.95818815331010454</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2021</v>
       </c>
@@ -2252,20 +2290,20 @@
         <f t="shared" si="1"/>
         <v>19.400000000000002</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="7">
         <f t="shared" si="2"/>
         <v>6.1855670103092772E-2</v>
       </c>
-      <c r="G7" s="10">
+      <c r="G7" s="26">
         <f t="shared" si="3"/>
         <v>5.1546391752577319E-3</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="8">
         <f t="shared" si="4"/>
         <v>0.9329896907216495</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2022</v>
       </c>
@@ -2282,20 +2320,20 @@
         <f t="shared" si="1"/>
         <v>21.3</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F8" s="7">
         <f t="shared" si="2"/>
         <v>8.9201877934272297E-2</v>
       </c>
-      <c r="G8" s="10">
+      <c r="G8" s="26">
         <f t="shared" si="3"/>
         <v>4.6948356807511738E-3</v>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="8">
         <f t="shared" si="4"/>
         <v>0.9061032863849765</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>2023</v>
       </c>
@@ -2312,20 +2350,20 @@
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="7">
         <f t="shared" si="2"/>
         <v>0.12608695652173912</v>
       </c>
-      <c r="G9" s="10">
+      <c r="G9" s="26">
         <f t="shared" si="3"/>
         <v>4.3478260869565218E-3</v>
       </c>
-      <c r="H9" s="11">
+      <c r="H9" s="8">
         <f t="shared" si="4"/>
         <v>0.86956521739130432</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2024</v>
       </c>
@@ -2342,20 +2380,20 @@
         <f t="shared" si="1"/>
         <v>25.2</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="7">
         <f t="shared" si="2"/>
         <v>0.15873015873015872</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="26">
         <f t="shared" si="3"/>
         <v>7.9365079365079378E-3</v>
       </c>
-      <c r="H10" s="11">
+      <c r="H10" s="8">
         <f t="shared" si="4"/>
         <v>0.83333333333333337</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>2025</v>
       </c>
@@ -2372,20 +2410,20 @@
         <f t="shared" si="1"/>
         <v>27.5</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="7">
         <f t="shared" si="2"/>
         <v>0.18909090909090909</v>
       </c>
-      <c r="G11" s="10">
+      <c r="G11" s="26">
         <f t="shared" si="3"/>
         <v>1.0909090909090908E-2</v>
       </c>
-      <c r="H11" s="11">
+      <c r="H11" s="8">
         <f t="shared" si="4"/>
         <v>0.8</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2026</v>
       </c>
@@ -2402,20 +2440,20 @@
         <f t="shared" si="1"/>
         <v>29.9</v>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="7">
         <f t="shared" si="2"/>
         <v>0.21404682274247494</v>
       </c>
-      <c r="G12" s="10">
+      <c r="G12" s="26">
         <f t="shared" si="3"/>
         <v>1.6722408026755852E-2</v>
       </c>
-      <c r="H12" s="11">
+      <c r="H12" s="8">
         <f t="shared" si="4"/>
         <v>0.76923076923076927</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>2027</v>
       </c>
@@ -2432,20 +2470,20 @@
         <f t="shared" si="1"/>
         <v>32.200000000000003</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="7">
         <f t="shared" si="2"/>
         <v>0.24223602484472048</v>
       </c>
-      <c r="G13" s="10">
+      <c r="G13" s="26">
         <f t="shared" si="3"/>
         <v>2.1739130434782605E-2</v>
       </c>
-      <c r="H13" s="11">
+      <c r="H13" s="8">
         <f t="shared" si="4"/>
         <v>0.73602484472049678</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>2028</v>
       </c>
@@ -2462,73 +2500,73 @@
         <f t="shared" si="1"/>
         <v>34.4</v>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="9">
         <f t="shared" si="2"/>
         <v>0.27325581395348841</v>
       </c>
-      <c r="G14" s="13">
+      <c r="G14" s="27">
         <f t="shared" si="3"/>
         <v>2.9069767441860465E-2</v>
       </c>
-      <c r="H14" s="14">
+      <c r="H14" s="10">
         <f t="shared" si="4"/>
         <v>0.69767441860465118</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="C15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="17"/>
+      <c r="D18" t="s">
         <v>64</v>
-      </c>
-      <c r="C18" s="4"/>
-      <c r="D18" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
-        <v>72</v>
-      </c>
-      <c r="C19" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>69</v>
       </c>
       <c r="D19" t="s">
-        <v>65</v>
-      </c>
-      <c r="E19" s="15" t="s">
-        <v>68</v>
+        <v>63</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>66</v>
       </c>
       <c r="F19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>2018</v>
       </c>
-      <c r="B20" s="5">
-        <f>C20/E20</f>
-        <v>2.3529411764705885E-3</v>
-      </c>
-      <c r="C20" s="15">
+      <c r="B20" s="28">
+        <f>C20/F20</f>
+        <v>3.1809145129224651E-5</v>
+      </c>
+      <c r="C20" s="11">
         <v>0.4</v>
       </c>
       <c r="D20">
         <v>4</v>
       </c>
-      <c r="E20" s="15">
+      <c r="E20" s="11">
         <v>170</v>
       </c>
       <c r="F20">
@@ -2539,17 +2577,17 @@
       <c r="A21">
         <v>2019</v>
       </c>
-      <c r="B21" s="5">
-        <f t="shared" ref="B21:B30" si="5">C21/E21</f>
-        <v>1.9138755980861245E-3</v>
-      </c>
-      <c r="C21" s="15">
+      <c r="B21" s="28">
+        <f t="shared" ref="B21:B30" si="5">C21/F21</f>
+        <v>3.0434451799436964E-5</v>
+      </c>
+      <c r="C21" s="11">
         <v>0.4</v>
       </c>
       <c r="D21">
         <v>9</v>
       </c>
-      <c r="E21" s="15">
+      <c r="E21" s="11">
         <v>209</v>
       </c>
       <c r="F21">
@@ -2560,17 +2598,17 @@
       <c r="A22">
         <v>2020</v>
       </c>
-      <c r="B22" s="5">
+      <c r="B22" s="28">
         <f t="shared" si="5"/>
-        <v>3.3018867924528299E-3</v>
-      </c>
-      <c r="C22" s="15">
+        <v>5.4192149880003095E-5</v>
+      </c>
+      <c r="C22" s="11">
         <v>0.7</v>
       </c>
       <c r="D22">
         <v>24</v>
       </c>
-      <c r="E22" s="15">
+      <c r="E22" s="11">
         <v>212</v>
       </c>
       <c r="F22">
@@ -2581,17 +2619,17 @@
       <c r="A23">
         <v>2021</v>
       </c>
-      <c r="B23" s="5">
+      <c r="B23" s="28">
         <f t="shared" si="5"/>
-        <v>3.8194444444444448E-3</v>
-      </c>
-      <c r="C23" s="15">
+        <v>8.058017727639001E-5</v>
+      </c>
+      <c r="C23" s="11">
         <v>1.1000000000000001</v>
       </c>
       <c r="D23">
         <v>66</v>
       </c>
-      <c r="E23" s="15">
+      <c r="E23" s="11">
         <v>288</v>
       </c>
       <c r="F23">
@@ -2602,17 +2640,17 @@
       <c r="A24">
         <v>2022</v>
       </c>
-      <c r="B24" s="5">
+      <c r="B24" s="28">
         <f t="shared" si="5"/>
-        <v>6.8459657701711489E-3</v>
-      </c>
-      <c r="C24" s="15">
+        <v>1.9553072625698323E-4</v>
+      </c>
+      <c r="C24" s="11">
         <v>2.8</v>
       </c>
       <c r="D24">
         <v>93</v>
       </c>
-      <c r="E24" s="15">
+      <c r="E24" s="11">
         <v>409</v>
       </c>
       <c r="F24">
@@ -2623,17 +2661,17 @@
       <c r="A25">
         <v>2023</v>
       </c>
-      <c r="B25" s="5">
+      <c r="B25" s="28">
         <f t="shared" si="5"/>
-        <v>9.6078431372549032E-3</v>
-      </c>
-      <c r="C25" s="15">
+        <v>3.3690869086908695E-4</v>
+      </c>
+      <c r="C25" s="11">
         <v>4.9000000000000004</v>
       </c>
       <c r="D25">
         <v>148</v>
       </c>
-      <c r="E25" s="15">
+      <c r="E25" s="11">
         <v>510</v>
       </c>
       <c r="F25">
@@ -2644,17 +2682,17 @@
       <c r="A26">
         <v>2024</v>
       </c>
-      <c r="B26" s="5">
+      <c r="B26" s="28">
         <f t="shared" si="5"/>
-        <v>1.2673611111111111E-2</v>
-      </c>
-      <c r="C26" s="15">
+        <v>4.8114948589506984E-4</v>
+      </c>
+      <c r="C26" s="11">
         <v>7.3</v>
       </c>
       <c r="D26">
         <v>183</v>
       </c>
-      <c r="E26" s="15">
+      <c r="E26" s="11">
         <v>576</v>
       </c>
       <c r="F26">
@@ -2665,17 +2703,17 @@
       <c r="A27">
         <v>2025</v>
       </c>
-      <c r="B27" s="5">
+      <c r="B27" s="28">
         <f t="shared" si="5"/>
-        <v>1.6773162939297124E-2</v>
-      </c>
-      <c r="C27" s="15">
+        <v>6.5715358618099887E-4</v>
+      </c>
+      <c r="C27" s="11">
         <v>10.5</v>
       </c>
       <c r="D27">
         <v>295</v>
       </c>
-      <c r="E27" s="15">
+      <c r="E27" s="11">
         <v>626</v>
       </c>
       <c r="F27">
@@ -2686,17 +2724,17 @@
       <c r="A28">
         <v>2026</v>
       </c>
-      <c r="B28" s="5">
+      <c r="B28" s="28">
         <f t="shared" si="5"/>
-        <v>2.2962962962962963E-2</v>
-      </c>
-      <c r="C28" s="15">
+        <v>9.1846409101682864E-4</v>
+      </c>
+      <c r="C28" s="11">
         <v>15.5</v>
       </c>
       <c r="D28">
         <v>482</v>
       </c>
-      <c r="E28" s="15">
+      <c r="E28" s="11">
         <v>675</v>
       </c>
       <c r="F28">
@@ -2707,17 +2745,17 @@
       <c r="A29">
         <v>2027</v>
       </c>
-      <c r="B29" s="5">
+      <c r="B29" s="28">
         <f t="shared" si="5"/>
-        <v>2.524271844660194E-2</v>
-      </c>
-      <c r="C29" s="15">
+        <v>1.028306683993446E-3</v>
+      </c>
+      <c r="C29" s="11">
         <v>18.2</v>
       </c>
       <c r="D29">
         <v>691</v>
       </c>
-      <c r="E29" s="15">
+      <c r="E29" s="11">
         <v>721</v>
       </c>
       <c r="F29">
@@ -2728,17 +2766,17 @@
       <c r="A30">
         <v>2028</v>
       </c>
-      <c r="B30" s="5">
+      <c r="B30" s="28">
         <f t="shared" si="5"/>
-        <v>2.8853754940711459E-2</v>
-      </c>
-      <c r="C30" s="15">
+        <v>1.1831442463533224E-3</v>
+      </c>
+      <c r="C30" s="11">
         <v>21.9</v>
       </c>
       <c r="D30">
         <v>991</v>
       </c>
-      <c r="E30" s="15">
+      <c r="E30" s="11">
         <v>759</v>
       </c>
       <c r="F30">
@@ -2761,78 +2799,78 @@
   <sheetData>
     <row r="1" spans="1:23" ht="17.5" x14ac:dyDescent="0.45">
       <c r="B1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="N1" t="s">
+        <v>46</v>
+      </c>
+      <c r="R1" t="s">
         <v>48</v>
       </c>
-      <c r="R1" t="s">
-        <v>50</v>
-      </c>
       <c r="V1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" t="s">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="s">
-        <v>24</v>
-      </c>
       <c r="E2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" t="s">
         <v>22</v>
       </c>
-      <c r="F2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G2" t="s">
-        <v>24</v>
-      </c>
       <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" t="s">
         <v>22</v>
       </c>
-      <c r="J2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" t="s">
-        <v>24</v>
-      </c>
       <c r="M2" t="s">
+        <v>20</v>
+      </c>
+      <c r="N2" t="s">
+        <v>21</v>
+      </c>
+      <c r="O2" t="s">
         <v>22</v>
       </c>
-      <c r="N2" t="s">
-        <v>23</v>
-      </c>
-      <c r="O2" t="s">
-        <v>24</v>
-      </c>
       <c r="Q2" t="s">
+        <v>20</v>
+      </c>
+      <c r="R2" t="s">
+        <v>21</v>
+      </c>
+      <c r="S2" t="s">
         <v>22</v>
       </c>
-      <c r="R2" t="s">
-        <v>23</v>
-      </c>
-      <c r="S2" t="s">
-        <v>24</v>
-      </c>
       <c r="U2" t="s">
+        <v>20</v>
+      </c>
+      <c r="V2" t="s">
+        <v>21</v>
+      </c>
+      <c r="W2" t="s">
         <v>22</v>
-      </c>
-      <c r="V2" t="s">
-        <v>23</v>
-      </c>
-      <c r="W2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.35">
@@ -2840,7 +2878,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C3">
         <v>0.30393992465576336</v>
@@ -2849,7 +2887,7 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G3">
         <v>0.90542979856308781</v>
@@ -2858,7 +2896,7 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="K3">
         <v>0.56331411719800495</v>
@@ -2867,7 +2905,7 @@
         <v>1</v>
       </c>
       <c r="N3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="O3">
         <v>0.31924702365464647</v>
@@ -2876,7 +2914,7 @@
         <v>1</v>
       </c>
       <c r="R3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S3">
         <v>0.36234318344008598</v>
@@ -2885,7 +2923,7 @@
         <v>1</v>
       </c>
       <c r="V3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="W3">
         <v>0.91452134589285305</v>
@@ -2896,7 +2934,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4">
         <v>0.18852060065724716</v>
@@ -2905,7 +2943,7 @@
         <v>2</v>
       </c>
       <c r="F4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G4">
         <v>4.1520674290600239E-2</v>
@@ -2914,7 +2952,7 @@
         <v>2</v>
       </c>
       <c r="J4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K4">
         <v>0.11678568072225042</v>
@@ -2923,7 +2961,7 @@
         <v>2</v>
       </c>
       <c r="N4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="O4">
         <v>0.23689856627905867</v>
@@ -2932,7 +2970,7 @@
         <v>2</v>
       </c>
       <c r="R4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="S4">
         <v>0.24172749055100812</v>
@@ -2941,7 +2979,7 @@
         <v>2</v>
       </c>
       <c r="V4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="W4">
         <v>4.8863343914320068E-2</v>
@@ -2952,7 +2990,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C5">
         <v>0.11614030403526776</v>
@@ -2961,7 +2999,7 @@
         <v>3</v>
       </c>
       <c r="F5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G5">
         <v>3.0331786784455011E-2</v>
@@ -2970,7 +3008,7 @@
         <v>3</v>
       </c>
       <c r="J5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="K5">
         <v>0.10788002212338918</v>
@@ -2979,7 +3017,7 @@
         <v>3</v>
       </c>
       <c r="N5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O5">
         <v>0.21584267751001046</v>
@@ -2988,7 +3026,7 @@
         <v>3</v>
       </c>
       <c r="R5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="S5">
         <v>0.1489190260820292</v>
@@ -2997,7 +3035,7 @@
         <v>3</v>
       </c>
       <c r="V5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="W5">
         <v>2.0395134851194461E-2</v>
@@ -3008,7 +3046,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C6">
         <v>0.10523141119195512</v>
@@ -3017,7 +3055,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G6">
         <v>2.2717740361856986E-2</v>
@@ -3026,7 +3064,7 @@
         <v>4</v>
       </c>
       <c r="J6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K6">
         <v>9.7508823924634447E-2</v>
@@ -3035,7 +3073,7 @@
         <v>4</v>
       </c>
       <c r="N6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O6">
         <v>0.10328875184219956</v>
@@ -3044,19 +3082,19 @@
         <v>4</v>
       </c>
       <c r="R6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="S6">
         <v>0.13493127470361002</v>
       </c>
       <c r="U6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="V6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="W6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.35">
@@ -3064,25 +3102,25 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C7">
         <v>7.2380296621979381E-2</v>
       </c>
       <c r="E7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I7">
         <v>5</v>
       </c>
       <c r="J7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="K7">
         <v>8.3074750800168254E-2</v>
@@ -3091,7 +3129,7 @@
         <v>5</v>
       </c>
       <c r="N7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="O7">
         <v>5.0258088334766339E-2</v>
@@ -3100,19 +3138,19 @@
         <v>5</v>
       </c>
       <c r="R7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="S7">
         <v>6.1163171426547702E-2</v>
       </c>
       <c r="U7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="V7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="W7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.35">
@@ -3120,25 +3158,25 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C8">
         <v>6.3315982871402013E-2</v>
       </c>
       <c r="E8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I8">
         <v>6</v>
       </c>
       <c r="J8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="K8">
         <v>3.1436605231552818E-2</v>
@@ -3147,7 +3185,7 @@
         <v>6</v>
       </c>
       <c r="N8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="O8">
         <v>4.1308401327102409E-2</v>
@@ -3156,19 +3194,19 @@
         <v>6</v>
       </c>
       <c r="R8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="S8">
         <v>2.5438294849965772E-2</v>
       </c>
       <c r="U8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="V8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="W8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.35">
@@ -3176,34 +3214,34 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C9">
         <v>5.3662117291731336E-2</v>
       </c>
       <c r="E9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="M9">
         <v>7</v>
       </c>
       <c r="N9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="O9">
         <v>2.8239042857085037E-2</v>
@@ -3212,19 +3250,19 @@
         <v>7</v>
       </c>
       <c r="R9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="S9">
         <v>2.5263049067487095E-2</v>
       </c>
       <c r="U9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="V9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="W9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.35">
@@ -3232,55 +3270,55 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C10">
         <v>3.1581866961590314E-2</v>
       </c>
       <c r="E10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="M10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="N10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="Q10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="R10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="U10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="V10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="W10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.35">
@@ -3288,55 +3326,55 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C11">
         <v>1.983904525662443E-2</v>
       </c>
       <c r="E11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="M11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="N11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="Q11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="R11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="U11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="V11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="W11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.35">
@@ -3344,258 +3382,258 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C12">
         <v>1.9702373005982925E-2</v>
       </c>
       <c r="E12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="M12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="N12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="Q12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="R12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="U12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="V12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="W12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="M13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="N13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="Q13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="R13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="U13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="V13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="W13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="M14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="N14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="Q14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="R14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="U14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="V14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="W14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="M15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="N15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="Q15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="R15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="U15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="V15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="W15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C16">
         <v>2.5686077450456257E-2</v>
       </c>
       <c r="F16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="N16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="R16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="V16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="W16">
         <v>1.6220175341632337E-2</v>
@@ -3603,37 +3641,37 @@
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C17">
         <v>48217.54210579193</v>
       </c>
       <c r="E17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G17">
         <v>3371.8142200714274</v>
       </c>
       <c r="I17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K17">
         <v>470.9481475798874</v>
       </c>
       <c r="M17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="O17">
         <v>4769.973992450834</v>
       </c>
       <c r="Q17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="S17">
         <v>37604.328656536789</v>
       </c>
       <c r="U17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="W17">
         <v>2000.4770891529802</v>
@@ -3645,15 +3683,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E1D7978D1E43DE4EA43DBD7340A406DC" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1d2a0579b8367a5d14f15657bceede69">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d382aed9-cc96-421a-b6d1-bad087b40ea5" xmlns:ns3="3c3bb480-5c86-45a4-be90-daa3829a93c5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6184784662eaf13c68ab2ee7ade41035" ns2:_="" ns3:_="">
     <xsd:import namespace="d382aed9-cc96-421a-b6d1-bad087b40ea5"/>
@@ -3896,6 +3925,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3909,14 +3947,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D15763B-BC3F-44A0-B84D-0D65F1925A17}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A8357D9-61C4-4864-BD66-2D2D973EC6D9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3931,6 +3961,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D15763B-BC3F-44A0-B84D-0D65F1925A17}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
updating baseline development files
mostly just tweaks, adding some things for REMADE TEA
</commit_message>
<xml_diff>
--- a/PV_ICE/baselines/SupportingMaterial/Manual Files/Inverter_Gallium_Calcs.xlsx
+++ b/PV_ICE/baselines/SupportingMaterial/Manual Files/Inverter_Gallium_Calcs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hmirletz\Documents\GitHub\PV_ICE\PV_ICE\baselines\SupportingMaterial\Manual Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9BC423E-1638-441F-9E90-A5B8A3074F98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C1366EB-F0EC-4CCD-815A-553FDFD7478A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Maths" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="864" uniqueCount="179">
   <si>
     <t>year</t>
   </si>
@@ -716,6 +716,9 @@
   </si>
   <si>
     <t>Utility [kg/MWac]</t>
+  </si>
+  <si>
+    <t>Large Non-Res ILR</t>
   </si>
 </sst>
 </file>
@@ -1685,6 +1688,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1692,7 +1696,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2622,7 +2625,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AG114"/>
+  <dimension ref="A1:AL114"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.81640625" bestFit="1" customWidth="1"/>
@@ -2908,7 +2911,7 @@
         <v>4.8503749441697556E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>2003</v>
       </c>
@@ -2922,7 +2925,7 @@
         <v>4.8503749441697556E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>2004</v>
       </c>
@@ -2936,7 +2939,7 @@
         <v>4.8503749441697556E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>2005</v>
       </c>
@@ -2950,7 +2953,7 @@
         <v>4.8503749441697556E-3</v>
       </c>
     </row>
-    <row r="20" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>2006</v>
       </c>
@@ -2964,7 +2967,7 @@
         <v>4.8503749441697556E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>2007</v>
       </c>
@@ -2978,7 +2981,7 @@
         <v>4.8503749441697556E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>2008</v>
       </c>
@@ -2992,7 +2995,7 @@
         <v>4.8503749441697556E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>2009</v>
       </c>
@@ -3005,8 +3008,11 @@
       <c r="AE23" s="41">
         <v>4.8503749441697556E-3</v>
       </c>
-    </row>
-    <row r="24" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI23" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="24" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>2010</v>
       </c>
@@ -3019,8 +3025,22 @@
       <c r="AE24" s="41">
         <v>4.8503749441697556E-3</v>
       </c>
-    </row>
-    <row r="25" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI24">
+        <v>2010.04157061054</v>
+      </c>
+      <c r="AJ24">
+        <v>1.02831858407079</v>
+      </c>
+      <c r="AK24">
+        <f>ROUND(AI24,0)</f>
+        <v>2010</v>
+      </c>
+      <c r="AL24">
+        <f>ROUND(AJ24,2)</f>
+        <v>1.03</v>
+      </c>
+    </row>
+    <row r="25" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>2011</v>
       </c>
@@ -3033,8 +3053,22 @@
       <c r="AE25" s="41">
         <v>4.8503749441697556E-3</v>
       </c>
-    </row>
-    <row r="26" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI25">
+        <v>2011.0358816092801</v>
+      </c>
+      <c r="AJ25">
+        <v>1.0893805309734399</v>
+      </c>
+      <c r="AK25">
+        <f t="shared" ref="AK25:AL37" si="0">ROUND(AI25,0)</f>
+        <v>2011</v>
+      </c>
+      <c r="AL25">
+        <f t="shared" ref="AL25:AL37" si="1">ROUND(AJ25,2)</f>
+        <v>1.0900000000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>2012</v>
       </c>
@@ -3047,8 +3081,22 @@
       <c r="AE26" s="41">
         <v>4.8503749441697556E-3</v>
       </c>
-    </row>
-    <row r="27" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI26">
+        <v>2012.07780545846</v>
+      </c>
+      <c r="AJ26">
+        <v>1.1119469026548601</v>
+      </c>
+      <c r="AK26">
+        <f t="shared" si="0"/>
+        <v>2012</v>
+      </c>
+      <c r="AL26">
+        <f t="shared" si="1"/>
+        <v>1.1100000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>2013</v>
       </c>
@@ -3061,8 +3109,22 @@
       <c r="AE27" s="41">
         <v>4.8503749441697556E-3</v>
       </c>
-    </row>
-    <row r="28" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI27">
+        <v>2013.09531865843</v>
+      </c>
+      <c r="AJ27">
+        <v>1.1504424778761</v>
+      </c>
+      <c r="AK27">
+        <f t="shared" si="0"/>
+        <v>2013</v>
+      </c>
+      <c r="AL27">
+        <f t="shared" si="1"/>
+        <v>1.1499999999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>2014</v>
       </c>
@@ -3081,8 +3143,22 @@
       <c r="AE28" s="41">
         <v>4.8503749441697556E-3</v>
       </c>
-    </row>
-    <row r="29" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI28">
+        <v>2014.0874544507999</v>
+      </c>
+      <c r="AJ28">
+        <v>1.1995575221238799</v>
+      </c>
+      <c r="AK28">
+        <f t="shared" si="0"/>
+        <v>2014</v>
+      </c>
+      <c r="AL28">
+        <f t="shared" si="1"/>
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>2015</v>
       </c>
@@ -3110,8 +3186,22 @@
         <f>WoodMacInverterCompany!V4</f>
         <v>4.8503749441697556E-3</v>
       </c>
-    </row>
-    <row r="30" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI29">
+        <v>2015.07282293448</v>
+      </c>
+      <c r="AJ29">
+        <v>1.2115044247787501</v>
+      </c>
+      <c r="AK29">
+        <f t="shared" si="0"/>
+        <v>2015</v>
+      </c>
+      <c r="AL29">
+        <f t="shared" si="1"/>
+        <v>1.21</v>
+      </c>
+    </row>
+    <row r="30" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>2016</v>
       </c>
@@ -3140,8 +3230,22 @@
         <f>WoodMacInverterCompany!V5</f>
         <v>5.7589593033124976E-3</v>
       </c>
-    </row>
-    <row r="31" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI30">
+        <v>2016.11716367963</v>
+      </c>
+      <c r="AJ30">
+        <v>1.24734513274335</v>
+      </c>
+      <c r="AK30">
+        <f t="shared" si="0"/>
+        <v>2016</v>
+      </c>
+      <c r="AL30">
+        <f t="shared" si="1"/>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>2017</v>
       </c>
@@ -3160,8 +3264,22 @@
         <f>WoodMacInverterCompany!V6</f>
         <v>2.8711770168524066E-3</v>
       </c>
-    </row>
-    <row r="32" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI31">
+        <v>2017.0728043429699</v>
+      </c>
+      <c r="AJ31">
+        <v>1.24601769911503</v>
+      </c>
+      <c r="AK31">
+        <f t="shared" si="0"/>
+        <v>2017</v>
+      </c>
+      <c r="AL31">
+        <f t="shared" si="1"/>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="32" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>2018</v>
       </c>
@@ -3186,7 +3304,7 @@
         <v>6.4508946322067582E-9</v>
       </c>
       <c r="W32" s="36">
-        <f t="shared" ref="W32:W37" si="0">$B$39*$G$38*$H$38*P32</f>
+        <f t="shared" ref="W32:W37" si="2">$B$39*$G$38*$H$38*P32</f>
         <v>1.9352683896620274E-8</v>
       </c>
       <c r="X32" s="27"/>
@@ -3219,8 +3337,22 @@
         <f>(Y32*AC32)+(Z32*AD32)+(AA32*AE32)</f>
         <v>5.3661361814351366E-9</v>
       </c>
-    </row>
-    <row r="33" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI32">
+        <v>2018.1350301182399</v>
+      </c>
+      <c r="AJ32">
+        <v>1.2300884955752101</v>
+      </c>
+      <c r="AK32">
+        <f t="shared" si="0"/>
+        <v>2018</v>
+      </c>
+      <c r="AL32">
+        <f t="shared" si="1"/>
+        <v>1.23</v>
+      </c>
+    </row>
+    <row r="33" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>2019</v>
       </c>
@@ -3241,11 +3373,11 @@
         <v>1.0286844708209693E-8</v>
       </c>
       <c r="V33" s="36">
-        <f t="shared" ref="V33:V42" si="1">$B$39*$G$36*P33</f>
+        <f t="shared" ref="V33:V42" si="3">$B$39*$G$36*P33</f>
         <v>6.1721068249258155E-9</v>
       </c>
       <c r="W33" s="36">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1.8516320474777446E-8</v>
       </c>
       <c r="X33" s="27"/>
@@ -3254,11 +3386,11 @@
         <v>6.4292779426310583E-9</v>
       </c>
       <c r="Z33" s="36">
-        <f t="shared" ref="Z33:Z42" si="2">V33/1000/$Z$1</f>
+        <f t="shared" ref="Z33:Z42" si="4">V33/1000/$Z$1</f>
         <v>6.1721068249258161E-10</v>
       </c>
       <c r="AA33" s="36">
-        <f t="shared" ref="AA33:AA42" si="3">W33/1000/$AA$1</f>
+        <f t="shared" ref="AA33:AA42" si="5">W33/1000/$AA$1</f>
         <v>1.8516320474777447E-11</v>
       </c>
       <c r="AB33" s="27"/>
@@ -3275,11 +3407,25 @@
         <v>3.7343167375427193E-3</v>
       </c>
       <c r="AG33" s="36">
-        <f t="shared" ref="AG33:AG42" si="4">(Y33*AC33)+(Z33*AD33)+(AA33*AE33)</f>
+        <f t="shared" ref="AG33:AG42" si="6">(Y33*AC33)+(Z33*AD33)+(AA33*AE33)</f>
         <v>5.3434114050482815E-9</v>
       </c>
-    </row>
-    <row r="34" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI33">
+        <v>2019.12088198111</v>
+      </c>
+      <c r="AJ33">
+        <v>1.24469026548672</v>
+      </c>
+      <c r="AK33">
+        <f t="shared" si="0"/>
+        <v>2019</v>
+      </c>
+      <c r="AL33">
+        <f t="shared" si="1"/>
+        <v>1.24</v>
+      </c>
+    </row>
+    <row r="34" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>2020</v>
       </c>
@@ -3296,28 +3442,28 @@
         <v>73</v>
       </c>
       <c r="U34" s="36">
-        <f t="shared" ref="U34:U42" si="5">$B$39*$G$37*P34</f>
+        <f t="shared" ref="U34:U42" si="7">$B$39*$G$37*P34</f>
         <v>1.8316946659441044E-8</v>
       </c>
       <c r="V34" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>1.0990167995664626E-8</v>
       </c>
       <c r="W34" s="36">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>3.2970503986993881E-8</v>
       </c>
       <c r="X34" s="27"/>
       <c r="Y34" s="36">
-        <f t="shared" ref="Y34:Y42" si="6">U34/1000/$Y$1</f>
+        <f t="shared" ref="Y34:Y42" si="8">U34/1000/$Y$1</f>
         <v>1.1448091662150651E-8</v>
       </c>
       <c r="Z34" s="36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1.0990167995664627E-9</v>
       </c>
       <c r="AA34" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.2970503986993881E-11</v>
       </c>
       <c r="AB34" s="27"/>
@@ -3334,11 +3480,25 @@
         <v>7.1361510773210171E-3</v>
       </c>
       <c r="AG34" s="36">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>9.5065958395668732E-9</v>
       </c>
-    </row>
-    <row r="35" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI34">
+        <v>2020.24111325946</v>
+      </c>
+      <c r="AJ34">
+        <v>1.24734513274335</v>
+      </c>
+      <c r="AK34">
+        <f t="shared" si="0"/>
+        <v>2020</v>
+      </c>
+      <c r="AL34">
+        <f t="shared" si="1"/>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>2021</v>
       </c>
@@ -3368,28 +3528,28 @@
         <v>73</v>
       </c>
       <c r="U35" s="36">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>2.7236099919419822E-8</v>
       </c>
       <c r="V35" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>1.6341659951651891E-8</v>
       </c>
       <c r="W35" s="36">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>4.9024979854955677E-8</v>
       </c>
       <c r="X35" s="27"/>
       <c r="Y35" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1.7022562449637387E-8</v>
       </c>
       <c r="Z35" s="36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1.6341659951651892E-9</v>
       </c>
       <c r="AA35" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>4.9024979854955678E-11</v>
       </c>
       <c r="AB35" s="27"/>
@@ -3406,11 +3566,25 @@
         <v>3.8070870635134027E-3</v>
       </c>
       <c r="AG35" s="36">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1.5031625680352174E-8</v>
       </c>
-    </row>
-    <row r="36" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI35">
+        <v>2021.1704097568199</v>
+      </c>
+      <c r="AJ35">
+        <v>1.25132743362831</v>
+      </c>
+      <c r="AK35">
+        <f t="shared" si="0"/>
+        <v>2021</v>
+      </c>
+      <c r="AL35">
+        <f t="shared" si="1"/>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="36" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>2022</v>
       </c>
@@ -3449,28 +3623,28 @@
         <v>73</v>
       </c>
       <c r="U36" s="36">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>6.6089385474860326E-8</v>
       </c>
       <c r="V36" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>3.9653631284916192E-8</v>
       </c>
       <c r="W36" s="36">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1.1896089385474858E-7</v>
       </c>
       <c r="X36" s="27"/>
       <c r="Y36" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>4.13058659217877E-8</v>
       </c>
       <c r="Z36" s="36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.9653631284916193E-9</v>
       </c>
       <c r="AA36" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.1896089385474859E-10</v>
       </c>
       <c r="AB36" s="27"/>
@@ -3487,11 +3661,25 @@
         <v>3.4344048825351459E-3</v>
       </c>
       <c r="AG36" s="36">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.723590270124415E-8</v>
       </c>
-    </row>
-    <row r="37" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI36">
+        <v>2022.0997062541801</v>
+      </c>
+      <c r="AJ36">
+        <v>1.25530973451326</v>
+      </c>
+      <c r="AK36">
+        <f t="shared" si="0"/>
+        <v>2022</v>
+      </c>
+      <c r="AL36">
+        <f t="shared" si="1"/>
+        <v>1.26</v>
+      </c>
+    </row>
+    <row r="37" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>2023</v>
       </c>
@@ -3530,28 +3718,28 @@
         <v>73</v>
       </c>
       <c r="U37" s="36">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1.1387513751375138E-7</v>
       </c>
       <c r="V37" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>6.8325082508250822E-8</v>
       </c>
       <c r="W37" s="36">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>2.0497524752475247E-7</v>
       </c>
       <c r="X37" s="27"/>
       <c r="Y37" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>7.1171960946094613E-8</v>
       </c>
       <c r="Z37" s="36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>6.8325082508250815E-9</v>
       </c>
       <c r="AA37" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.0497524752475247E-10</v>
       </c>
       <c r="AB37" s="27"/>
@@ -3568,11 +3756,25 @@
         <v>9.5944618750836153E-3</v>
       </c>
       <c r="AG37" s="36">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>6.1887715743716504E-8</v>
       </c>
-    </row>
-    <row r="38" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AI37">
+        <v>2023.10972707667</v>
+      </c>
+      <c r="AJ37">
+        <v>1.25265486725663</v>
+      </c>
+      <c r="AK37">
+        <f t="shared" si="0"/>
+        <v>2023</v>
+      </c>
+      <c r="AL37">
+        <f t="shared" si="1"/>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="38" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>2024</v>
       </c>
@@ -3626,11 +3828,11 @@
         <v>73</v>
       </c>
       <c r="U38" s="36">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1.6262852623253359E-7</v>
       </c>
       <c r="V38" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>9.7577115739520148E-8</v>
       </c>
       <c r="W38" s="36">
@@ -3639,15 +3841,15 @@
       </c>
       <c r="X38" s="27"/>
       <c r="Y38" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1.016428288953335E-7</v>
       </c>
       <c r="Z38" s="36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>9.7577115739520142E-9</v>
       </c>
       <c r="AA38" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.9273134721856047E-10</v>
       </c>
       <c r="AB38" s="27"/>
@@ -3661,11 +3863,11 @@
         <v>9.5944618750836153E-3</v>
       </c>
       <c r="AG38" s="36">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>8.8383717666933081E-8</v>
       </c>
     </row>
-    <row r="39" spans="1:33" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:38" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>2025</v>
       </c>
@@ -3709,28 +3911,28 @@
         <v>73</v>
       </c>
       <c r="U39" s="37">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>2.2211791212917761E-7</v>
       </c>
       <c r="V39" s="37">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>1.3327074727750656E-7</v>
       </c>
       <c r="W39" s="36">
-        <f t="shared" ref="W39:W42" si="7">$B$39*$G$38*$H$38*P39</f>
+        <f t="shared" ref="W39:W42" si="9">$B$39*$G$38*$H$38*P39</f>
         <v>3.9981224183251968E-7</v>
       </c>
       <c r="X39" s="35"/>
       <c r="Y39" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1.3882369508073601E-7</v>
       </c>
       <c r="Z39" s="36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1.3327074727750655E-8</v>
       </c>
       <c r="AA39" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.9981224183251968E-10</v>
       </c>
       <c r="AB39" s="27"/>
@@ -3744,11 +3946,11 @@
         <v>9.5944618750836153E-3</v>
       </c>
       <c r="AG39" s="36">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1.207144114822988E-7</v>
       </c>
     </row>
-    <row r="40" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>2026</v>
       </c>
@@ -3765,28 +3967,28 @@
         <v>73</v>
       </c>
       <c r="U40" s="36">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>3.1044086276368805E-7</v>
       </c>
       <c r="V40" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>1.8626451765821281E-7</v>
       </c>
       <c r="W40" s="36">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>5.5879355297463852E-7</v>
       </c>
       <c r="X40" s="27"/>
       <c r="Y40" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1.9402553922730501E-7</v>
       </c>
       <c r="Z40" s="36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1.862645176582128E-8</v>
       </c>
       <c r="AA40" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>5.5879355297463856E-10</v>
       </c>
       <c r="AB40" s="27"/>
@@ -3800,11 +4002,11 @@
         <v>9.5944618750836153E-3</v>
       </c>
       <c r="AG40" s="36">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1.6871528139874396E-7</v>
       </c>
     </row>
-    <row r="41" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>2027</v>
       </c>
@@ -3821,28 +4023,28 @@
         <v>73</v>
       </c>
       <c r="U41" s="36">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>3.4756765918978473E-7</v>
       </c>
       <c r="V41" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>2.085405955138708E-7</v>
       </c>
       <c r="W41" s="36">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>6.2562178654161249E-7</v>
       </c>
       <c r="X41" s="27"/>
       <c r="Y41" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>2.1722978699361545E-7</v>
       </c>
       <c r="Z41" s="36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2.085405955138708E-8</v>
       </c>
       <c r="AA41" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>6.2562178654161252E-10</v>
       </c>
       <c r="AB41" s="27"/>
@@ -3856,11 +4058,11 @@
         <v>9.5944618750836153E-3</v>
       </c>
       <c r="AG41" s="36">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1.8889257974374607E-7</v>
       </c>
     </row>
-    <row r="42" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>2028</v>
       </c>
@@ -3877,28 +4079,28 @@
         <v>73</v>
       </c>
       <c r="U42" s="36">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>3.9990275526742293E-7</v>
       </c>
       <c r="V42" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>2.3994165316045375E-7</v>
       </c>
       <c r="W42" s="36">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>7.1982495948136129E-7</v>
       </c>
       <c r="X42" s="27"/>
       <c r="Y42" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>2.4993922204213932E-7</v>
       </c>
       <c r="Z42" s="36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2.3994165316045373E-8</v>
       </c>
       <c r="AA42" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>7.1982495948136124E-10</v>
       </c>
       <c r="AB42" s="27"/>
@@ -3912,11 +4114,11 @@
         <v>9.5944618750836153E-3</v>
       </c>
       <c r="AG42" s="36">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.1733513200043898E-7</v>
       </c>
     </row>
-    <row r="43" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>2029</v>
       </c>
@@ -3930,7 +4132,7 @@
         <v>9.5944618750836153E-3</v>
       </c>
     </row>
-    <row r="44" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>2030</v>
       </c>
@@ -3944,7 +4146,7 @@
         <v>9.5944618750836153E-3</v>
       </c>
     </row>
-    <row r="45" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>2031</v>
       </c>
@@ -3958,7 +4160,7 @@
         <v>9.5944618750836153E-3</v>
       </c>
     </row>
-    <row r="46" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>2032</v>
       </c>
@@ -3972,7 +4174,7 @@
         <v>9.5944618750836153E-3</v>
       </c>
     </row>
-    <row r="47" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>2033</v>
       </c>
@@ -3986,7 +4188,7 @@
         <v>9.5944618750836153E-3</v>
       </c>
     </row>
-    <row r="48" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>2034</v>
       </c>
@@ -10666,6 +10868,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <ProcessName xmlns="d382aed9-cc96-421a-b6d1-bad087b40ea5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d382aed9-cc96-421a-b6d1-bad087b40ea5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="3c3bb480-5c86-45a4-be90-daa3829a93c5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E1D7978D1E43DE4EA43DBD7340A406DC" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1d2a0579b8367a5d14f15657bceede69">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d382aed9-cc96-421a-b6d1-bad087b40ea5" xmlns:ns3="3c3bb480-5c86-45a4-be90-daa3829a93c5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6184784662eaf13c68ab2ee7ade41035" ns2:_="" ns3:_="">
     <xsd:import namespace="d382aed9-cc96-421a-b6d1-bad087b40ea5"/>
@@ -10908,28 +11131,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2355CD45-2F25-4965-9590-C756C8D0B153}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3c3bb480-5c86-45a4-be90-daa3829a93c5"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="d382aed9-cc96-421a-b6d1-bad087b40ea5"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <ProcessName xmlns="d382aed9-cc96-421a-b6d1-bad087b40ea5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d382aed9-cc96-421a-b6d1-bad087b40ea5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="3c3bb480-5c86-45a4-be90-daa3829a93c5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D15763B-BC3F-44A0-B84D-0D65F1925A17}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A8357D9-61C4-4864-BD66-2D2D973EC6D9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10948,31 +11175,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D15763B-BC3F-44A0-B84D-0D65F1925A17}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2355CD45-2F25-4965-9590-C756C8D0B153}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3c3bb480-5c86-45a4-be90-daa3829a93c5"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="d382aed9-cc96-421a-b6d1-bad087b40ea5"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{95965d95-ecc0-4720-b759-1f33c42ed7da}" enabled="1" method="Standard" siteId="{a0f29d7e-28cd-4f54-8442-7885aee7c080}" removed="0"/>

</xml_diff>